<commit_message>
chore(magazines): append JEE Main 2027 Session 1 entry
</commit_message>
<xml_diff>
--- a/career-magazines/CompetitionSuccessReview_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/CompetitionSuccessReview_Log_Apr2025-Sep2026.xlsx
@@ -162,7 +162,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -256,6 +256,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -689,7 +692,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 28 September 2026 | updated 24 October 2026 with the 1-24 October 2026 scrape</t>
+          <t>Compiled 26 October 2026 | updated automatically on each scheduled refresh. Sections: scholarships &amp; fellowships, internships, admissions / entrance exams (government job recruitment excluded).</t>
         </is>
       </c>
     </row>
@@ -733,8 +736,6 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="17"/>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="17">
       <c r="B17" s="20" t="inlineStr">
         <is>
@@ -807,7 +808,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="17">
       <c r="B23" s="26" t="inlineStr">
         <is>
@@ -821,10 +821,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B9:D10"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
+    <mergeCell ref="B11:D12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -3072,89 +3072,176 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Admission / Entrance Exam</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>SWAYAM-2026 (July Semester) Examination - 662 courses</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>National Testing Agency (NTA), Ministry of Education</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Candidates enrolled in SWAYAM online courses (UG/PG level) seeking proctored end-semester certification</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>No age limit prescribed</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="16" t="inlineStr">
         <is>
           <t>Twice-yearly (January and July semesters)</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="16" t="inlineStr">
         <is>
           <t>SWAYAM course credit / certification examination; exam fee as per the NTA information bulletin</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="16" t="inlineStr">
         <is>
           <t>Applications 09-10-2026 to 31-10-2026 (exam 08-12-2026 to 12-12-2026)</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M27" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N27" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O27" s="16" t="inlineStr">
         <is>
           <t>https://exams.nta.nic.in/swayam/</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" s="16" t="inlineStr">
         <is>
           <t>https://nta.ac.in/Download/Notice/Notice_20261009123259.pdf</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" s="16" t="inlineStr">
         <is>
           <t>NTA public notice dated 09 October 2026. Included as CSR-type NTA entrance/exam coverage; the specific CSR issue placement was not directly verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>JEE (Main) 2027 - Session 1 (January 2027)</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>National Testing Agency (NTA) for the Department of Higher Education, Ministry of Education</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>Class 12 students and pass-outs - Paper 1 for B.E./B.Tech admission at NITs, IIITs and other centrally funded technical institutions; Paper 2A/2B for B.Arch and B.Planning; also the eligibility test for JEE (Advanced)</t>
+        </is>
+      </c>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t>All categories (examination fee varies by category; Gen-EWS/OBC-NCL and SC/ST/PwD pay the reduced fee)</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I28" s="32" t="inlineStr">
+        <is>
+          <t>No age range prescribed in the public notice - eligibility is fixed by the year of passing the Class 12 qualifying examination</t>
+        </is>
+      </c>
+      <c r="J28" s="32" t="inlineStr">
+        <is>
+          <t>Annual, two sessions (Session 1 January 2027; Session 2 April 2027)</t>
+        </is>
+      </c>
+      <c r="K28" s="32" t="inlineStr">
+        <is>
+          <t>Gateway to NITs, IIITs and CFTIs and the eligibility test for JEE (Advanced); examination fee as per the NTA Information Bulletin (additional Rs 500 late fee outside the main window)</t>
+        </is>
+      </c>
+      <c r="L28" s="32" t="inlineStr">
+        <is>
+          <t>Applications 24.10.2026 to 22.11.2026 (11:50 PM); late-fee window 23.11.2026 to 26.11.2026; correction 27-29.11.2026; city slip 30.12.2026; admit cards 13.01.2027; exam 20, 21, 22, 23, 24 and 28.01.2027</t>
+        </is>
+      </c>
+      <c r="M28" s="32" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="N28" s="32" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O28" s="32" t="inlineStr">
+        <is>
+          <t>jeemain.nta.nic.in</t>
+        </is>
+      </c>
+      <c r="P28" s="32" t="inlineStr">
+        <is>
+          <t>https://nta.ac.in/Download/Notice/Notice_20261024220013.pdf ; https://www.competitionreview.in/</t>
+        </is>
+      </c>
+      <c r="Q28" s="32" t="inlineStr">
+        <is>
+          <t>The current CSR issue carries the cover feature "JEE Main 2027 - How to Score 99 Percentile"; application and examination dates are taken from NTA's public notice dated 24.10.2026 and the JEE (Main) 2027 Information Bulletin</t>
         </is>
       </c>
     </row>

</xml_diff>